<commit_message>
Collecte SCPI automatique 2026-09-14
</commit_message>
<xml_diff>
--- a/SCPI_tracker.xlsx
+++ b/SCPI_tracker.xlsx
@@ -19,8 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparatif'!$A$1:$P$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sources'!$A$1:$H$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'A_VERIFIER'!$A$1:$E$234</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Portefeuille'!$A$3:$Q$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +54,10 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,10 +100,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2224,71 +2228,19 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Mon portefeuille</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Montant investi</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>16200</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Valeur courante</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>17570</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>+/- value latente</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1370</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Dividendes encaissés</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>137.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>TRI global (XIRR)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>3.11 %</t>
+          <t>Vue portefeuille vide : copiez portefeuille.example.yaml en portefeuille.yaml pour l'alimenter.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Couverture des données</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>SCPI suivies</t>
         </is>
@@ -2298,39 +2250,39 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Métriques OK</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>75</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>À vérifier</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>233</v>
+        <v>466</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Taux de distribution par SCPI</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>SCPI</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>TD %</t>
         </is>
@@ -2490,89 +2442,89 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>SCPI</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Société de gestion</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Prix souscription</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Prix retrait</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Val. reconstitution</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Val. réalisation</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Écart prix/reconst.</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>TD</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>TRI 5 ans</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>TRI 10 ans</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>TOF</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Capitalisation</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Associés</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>Immeubles</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
         <is>
           <t>Délai jouiss.</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>Frais gestion</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>ActivImmo</t>
         </is>
@@ -2588,7 +2540,7 @@
       <c r="D2" t="n">
         <v>548.47</v>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2596,22 +2548,22 @@
       <c r="F2" t="n">
         <v>507.98</v>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2619,12 +2571,12 @@
       <c r="K2" t="n">
         <v>93.3</v>
       </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M2" s="7" t="n">
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="n">
         <v>29843</v>
       </c>
       <c r="N2" t="n">
@@ -2633,14 +2585,14 @@
       <c r="O2" t="n">
         <v>6</v>
       </c>
-      <c r="P2" s="6" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Comète</t>
         </is>
@@ -2656,7 +2608,7 @@
       <c r="D3" t="n">
         <v>225</v>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2664,7 +2616,7 @@
       <c r="F3" t="n">
         <v>217.17</v>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2672,32 +2624,32 @@
       <c r="H3" t="n">
         <v>6</v>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2705,14 +2657,14 @@
       <c r="O3" t="n">
         <v>6</v>
       </c>
-      <c r="P3" s="6" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>MomenTime</t>
         </is>
@@ -2722,47 +2674,47 @@
           <t>Arkéa Real Estate Investment Management</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2770,12 +2722,12 @@
       <c r="L4" t="n">
         <v>48800000</v>
       </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2788,7 +2740,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Transitions Europe</t>
         </is>
@@ -2798,7 +2750,7 @@
           <t>Arkéa Real Estate Investment Management</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2806,37 +2758,37 @@
       <c r="D5" t="n">
         <v>181.8</v>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2844,12 +2796,12 @@
       <c r="L5" t="n">
         <v>1380000000</v>
       </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2862,7 +2814,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Corum Eurion</t>
         </is>
@@ -2872,10 +2824,10 @@
           <t>Corum L'Épargne</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>215</v>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2886,23 +2838,23 @@
       <c r="F6" t="n">
         <v>177.1</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="8" t="n">
         <v>-3.21</v>
       </c>
       <c r="H6" t="n">
         <v>5.73</v>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -2910,27 +2862,27 @@
       <c r="L6" t="n">
         <v>1534000000</v>
       </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N6" s="7" t="n">
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="O6" s="6" t="inlineStr">
+      <c r="O6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P6" s="6" t="inlineStr">
+      <c r="P6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Corum Origin</t>
         </is>
@@ -2940,79 +2892,79 @@
           <t>Corum L'Épargne</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O7" s="6" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P7" s="6" t="inlineStr">
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Corum USA</t>
         </is>
@@ -3022,10 +2974,10 @@
           <t>Corum L'Épargne</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3036,23 +2988,23 @@
       <c r="F8" t="n">
         <v>177.04</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <v>-1.59</v>
       </c>
       <c r="H8" t="n">
         <v>7.7</v>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3060,27 +3012,27 @@
       <c r="L8" t="n">
         <v>77000000</v>
       </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N8" s="7" t="n">
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O8" s="6" t="inlineStr">
+      <c r="O8" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
+      <c r="P8" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Corum XL</t>
         </is>
@@ -3090,79 +3042,79 @@
           <t>Corum L'Épargne</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P9" s="6" t="inlineStr">
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Selectipierre 2</t>
         </is>
@@ -3172,7 +3124,7 @@
           <t>Fiducial Gérance</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3180,32 +3132,32 @@
       <c r="D10" t="n">
         <v>695.7</v>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3213,17 +3165,17 @@
       <c r="K10" t="n">
         <v>95.05</v>
       </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3231,14 +3183,14 @@
       <c r="O10" t="n">
         <v>2</v>
       </c>
-      <c r="P10" s="6" t="inlineStr">
+      <c r="P10" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Cristal Life</t>
         </is>
@@ -3248,47 +3200,47 @@
           <t>Inter Gestion REIM</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3296,29 +3248,29 @@
       <c r="L11" t="n">
         <v>424000000</v>
       </c>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O11" s="6" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P11" s="6" t="inlineStr">
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Cristal Rente</t>
         </is>
@@ -3331,32 +3283,32 @@
       <c r="C12" t="n">
         <v>255.68</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3364,7 +3316,7 @@
       <c r="J12" t="n">
         <v>5.56</v>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3372,29 +3324,29 @@
       <c r="L12" t="n">
         <v>684000000</v>
       </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O12" s="6" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O12" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P12" s="6" t="inlineStr">
+      <c r="P12" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Kyaneos Denormandie 5</t>
         </is>
@@ -3404,79 +3356,79 @@
           <t>Kyaneos Asset Management</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Kyaneos Pierre</t>
         </is>
@@ -3489,42 +3441,42 @@
       <c r="C14" t="n">
         <v>224</v>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3532,10 +3484,10 @@
       <c r="L14" t="n">
         <v>453000000</v>
       </c>
-      <c r="M14" s="7" t="n">
+      <c r="M14" s="8" t="n">
         <v>11091</v>
       </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3543,14 +3495,14 @@
       <c r="O14" t="n">
         <v>6</v>
       </c>
-      <c r="P14" s="6" t="inlineStr">
+      <c r="P14" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Fair Invest</t>
         </is>
@@ -3563,22 +3515,22 @@
       <c r="C15" t="n">
         <v>202</v>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3589,12 +3541,12 @@
       <c r="I15" t="n">
         <v>2.87</v>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3602,29 +3554,29 @@
       <c r="L15" t="n">
         <v>118700000</v>
       </c>
-      <c r="M15" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O15" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P15" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>NCap Continent</t>
         </is>
@@ -3637,22 +3589,22 @@
       <c r="C16" t="n">
         <v>210</v>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3660,17 +3612,17 @@
       <c r="H16" t="n">
         <v>7.1</v>
       </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3678,29 +3630,29 @@
       <c r="L16" t="n">
         <v>81500000</v>
       </c>
-      <c r="M16" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P16" s="6" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>NCap Régions</t>
         </is>
@@ -3713,22 +3665,22 @@
       <c r="C17" t="n">
         <v>682</v>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3739,12 +3691,12 @@
       <c r="I17" t="n">
         <v>5.44</v>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -3752,29 +3704,29 @@
       <c r="L17" t="n">
         <v>1106700000</v>
       </c>
-      <c r="M17" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N17" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O17" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P17" s="6" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>PF Grand Paris</t>
         </is>
@@ -3784,77 +3736,77 @@
           <t>Perial Asset Management</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="H18" s="8" t="n">
         <v>4.8</v>
       </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O18" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P18" s="6" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>PF Hospitalité Europe</t>
         </is>
@@ -3864,77 +3816,77 @@
           <t>Perial Asset Management</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H19" s="7" t="n">
+      <c r="H19" s="8" t="n">
         <v>4.11</v>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P19" s="6" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>PFO</t>
         </is>
@@ -3944,77 +3896,77 @@
           <t>Perial Asset Management</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="H20" s="8" t="n">
         <v>6.1</v>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>PFO2</t>
         </is>
@@ -4024,77 +3976,77 @@
           <t>Perial Asset Management</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H21" s="7" t="n">
+      <c r="H21" s="8" t="n">
         <v>4.65</v>
       </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P21" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Immorente</t>
         </is>
@@ -4104,79 +4056,79 @@
           <t>Sofidy</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P22" s="6" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Sofidy Europe Invest</t>
         </is>
@@ -4186,79 +4138,79 @@
           <t>Sofidy</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="O23" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="P23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Cœur d'Avenir</t>
         </is>
@@ -4274,52 +4226,52 @@
       <c r="D24" t="n">
         <v>180</v>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N24" s="5" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -4327,14 +4279,14 @@
       <c r="O24" t="n">
         <v>6</v>
       </c>
-      <c r="P24" s="6" t="inlineStr">
+      <c r="P24" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Cœur d'Europe</t>
         </is>
@@ -4350,17 +4302,17 @@
       <c r="D25" t="n">
         <v>179.52</v>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4371,25 +4323,25 @@
       <c r="I25" t="n">
         <v>3.46</v>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L25" s="7" t="n">
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="n">
         <v>275400000</v>
       </c>
-      <c r="M25" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N25" s="5" t="inlineStr">
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N25" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -4397,14 +4349,14 @@
       <c r="O25" t="n">
         <v>6</v>
       </c>
-      <c r="P25" s="6" t="inlineStr">
+      <c r="P25" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Cœur de Régions</t>
         </is>
@@ -4420,17 +4372,17 @@
       <c r="D26" t="n">
         <v>584.3200000000001</v>
       </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4441,25 +4393,25 @@
       <c r="I26" t="n">
         <v>4.44</v>
       </c>
-      <c r="J26" s="6" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="L26" s="7" t="n">
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="n">
         <v>441400000</v>
       </c>
-      <c r="M26" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="N26" s="5" t="inlineStr">
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="N26" s="6" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
         </is>
@@ -4467,7 +4419,7 @@
       <c r="O26" t="n">
         <v>6</v>
       </c>
-      <c r="P26" s="6" t="inlineStr">
+      <c r="P26" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4584,42 +4536,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>SCPI</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Métrique</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Période</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Date publication</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Confiance</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Source (URL)</t>
         </is>
@@ -7348,27 +7300,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>SCPI</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Métrique</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Période</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Raison</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Lien direct</t>
         </is>
@@ -12787,7 +12739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12800,37 +12752,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>SCPI</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Métrique</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Période</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Date publication</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Date collecte</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Confiance</t>
         </is>
@@ -12869,7 +12821,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>coeur_davenir</t>
+          <t>activimmo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12878,7 +12830,12 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>200</v>
+        <v>613.5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -12894,7 +12851,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12903,12 +12860,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>664</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -12924,26 +12876,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -12959,7 +12901,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -12968,7 +12910,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>204</v>
+        <v>664</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -12989,21 +12931,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6.25</v>
+        <v>664</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -13024,16 +12961,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>250</v>
+        <v>6.2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -13054,7 +12996,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -13068,7 +13010,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -13089,21 +13031,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>acompte</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2.75</v>
+        <v>204</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -13124,7 +13061,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -13132,13 +13069,8 @@
           <t>prix_souscription</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
-        </is>
-      </c>
       <c r="D11" t="n">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -13152,14 +13084,14 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -13173,7 +13105,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5.73</v>
+        <v>6.25</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -13194,21 +13126,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>200</v>
+        <v>6.25</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -13222,28 +13154,23 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>7.7</v>
+        <v>250</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -13264,7 +13191,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -13273,7 +13200,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>255.68</v>
+        <v>250</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -13294,16 +13221,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>202</v>
+        <v>6</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -13324,7 +13256,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -13338,7 +13270,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4.52</v>
+        <v>6</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -13359,16 +13291,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>224</v>
+        <v>2.75</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -13389,16 +13326,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>210</v>
+        <v>2.75</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -13419,21 +13361,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>7.1</v>
+        <v>215</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -13447,14 +13389,14 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -13462,8 +13404,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D21" t="n">
-        <v>682</v>
+        <v>215</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -13477,14 +13424,14 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -13498,7 +13445,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>7.51</v>
+        <v>5.73</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -13519,7 +13466,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -13533,7 +13480,12 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4.8</v>
+        <v>5.73</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -13542,28 +13494,33 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>4.11</v>
+        <v>200</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -13579,21 +13536,26 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6.1</v>
+        <v>200</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -13609,35 +13571,825 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>corum_usa</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>corum_usa</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cristal_rente</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>255.68</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>cristal_rente</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>255.68</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>fair_invest</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>202</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fair_invest</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>202</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fair_invest</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fair_invest</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>kyaneos_pierre</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>224</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>kyaneos_pierre</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>224</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>210</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>210</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>682</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>682</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>pfo2</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>taux_distribution</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D50" t="n">
         <v>4.65</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:G51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13648,7 +14400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13660,32 +14412,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>SCPI</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Période</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Acompte / part</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Date publication</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Confiance</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -13716,6 +14468,36 @@
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>corum_eurion</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
         </is>
@@ -13732,27 +14514,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -13762,283 +14525,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>SCPI</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Date achat</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Nb parts</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Prix unit.</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Frais</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Détention</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Démemb. (ans)</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Investi</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>PRU</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Prix courant</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>Valeur courante</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>+/- value latente</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Dividendes</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>Rendt/coût %</t>
-        </is>
-      </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>TRI réel %</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>corum_eurion</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2024-01-15</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" t="n">
-        <v>200</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>pleine</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>direct</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J4" t="n">
-        <v>200</v>
-      </c>
-      <c r="K4" t="n">
-        <v>215</v>
-      </c>
-      <c r="L4" t="n">
-        <v>10750</v>
-      </c>
-      <c r="M4" t="n">
-        <v>750</v>
-      </c>
-      <c r="N4" t="n">
-        <v>137.5</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="P4" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="Q4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ncap_regions</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2023-06-01</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D5" t="n">
-        <v>620</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>pleine</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>AV</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>6200</v>
-      </c>
-      <c r="J5" t="n">
-        <v>620</v>
-      </c>
-      <c r="K5" t="n">
-        <v>682</v>
-      </c>
-      <c r="L5" t="n">
-        <v>6820</v>
-      </c>
-      <c r="M5" t="n">
-        <v>620</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>2.94</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Acomptes non collectés — dividendes/TRI partiels (voir A_VERIFIER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>comete</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2025-03-10</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>40</v>
-      </c>
-      <c r="D6" t="n">
-        <v>250</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nue</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>7</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>direct</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J6" t="n">
-        <v>250</v>
-      </c>
-      <c r="K6" t="n">
-        <v>225</v>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>À VÉRIFIER</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Nue-propriété : aucun dividende pendant le démembrement ; valorisation nécessite une clé de démembrement (non calculée)</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Aucune ligne : copiez portefeuille.example.yaml en portefeuille.yaml.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:Q6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Collecte SCPI automatique 2026-09-15
</commit_message>
<xml_diff>
--- a/SCPI_tracker.xlsx
+++ b/SCPI_tracker.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparatif'!$A$1:$P$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sources'!$A$1:$H$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'A_VERIFIER'!$A$1:$E$234</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>150</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>466</v>
+        <v>699</v>
       </c>
     </row>
     <row r="16">
@@ -12739,7 +12739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12851,7 +12851,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>coeur_davenir</t>
+          <t>activimmo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12860,11 +12860,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>613.5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -12901,7 +12906,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -12910,12 +12915,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>664</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -12931,7 +12931,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -12940,16 +12940,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>664</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -12966,16 +12961,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -13001,16 +12991,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -13031,7 +13016,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -13040,7 +13025,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>204</v>
+        <v>664</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -13049,7 +13034,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -13061,16 +13046,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -13091,7 +13081,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -13105,7 +13095,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6.25</v>
+        <v>6.2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -13126,7 +13116,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -13140,7 +13130,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6.25</v>
+        <v>6.2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -13149,7 +13139,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -13161,7 +13151,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -13170,7 +13160,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -13191,7 +13181,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -13200,7 +13190,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -13221,21 +13211,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>204</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -13244,7 +13229,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -13256,7 +13241,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -13270,7 +13255,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -13291,21 +13276,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2.75</v>
+        <v>6.25</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -13326,21 +13311,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2.75</v>
+        <v>6.25</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -13349,7 +13334,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -13361,7 +13346,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -13369,13 +13354,8 @@
           <t>prix_souscription</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
-        </is>
-      </c>
       <c r="D20" t="n">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -13389,14 +13369,14 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -13404,13 +13384,8 @@
           <t>prix_souscription</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
-        </is>
-      </c>
       <c r="D21" t="n">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -13424,28 +13399,23 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5.73</v>
+        <v>250</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -13454,7 +13424,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -13466,7 +13436,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -13480,7 +13450,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5.73</v>
+        <v>6</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -13501,21 +13471,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>200</v>
+        <v>6</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -13529,28 +13499,28 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>200</v>
+        <v>6</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -13559,33 +13529,33 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7.7</v>
+        <v>2.75</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -13606,21 +13576,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7.7</v>
+        <v>2.75</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -13641,16 +13611,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>255.68</v>
+        <v>2.75</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -13659,7 +13634,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -13671,7 +13646,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -13679,8 +13654,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D29" t="n">
-        <v>255.68</v>
+        <v>215</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -13694,14 +13674,14 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -13709,8 +13689,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D30" t="n">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -13724,14 +13709,14 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -13739,8 +13724,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D31" t="n">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -13749,19 +13739,19 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -13775,7 +13765,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>4.52</v>
+        <v>5.73</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -13796,7 +13786,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -13810,7 +13800,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>4.52</v>
+        <v>5.73</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -13831,16 +13821,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>224</v>
+        <v>5.73</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -13849,7 +13844,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -13861,7 +13856,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -13869,8 +13864,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D35" t="n">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -13884,14 +13884,14 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -13899,8 +13899,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D36" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -13914,14 +13919,14 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -13929,8 +13934,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D37" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -13939,19 +13949,19 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -13965,7 +13975,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -13986,7 +13996,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -14000,7 +14010,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -14021,16 +14031,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>682</v>
+        <v>7.7</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -14039,7 +14054,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -14051,7 +14066,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -14060,7 +14075,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>682</v>
+        <v>255.68</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -14081,21 +14096,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>7.51</v>
+        <v>255.68</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -14116,21 +14126,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>7.51</v>
+        <v>255.68</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -14139,7 +14144,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -14151,21 +14156,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>4.8</v>
+        <v>202</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -14174,28 +14179,28 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>4.8</v>
+        <v>202</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -14204,44 +14209,44 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.11</v>
+        <v>202</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -14255,7 +14260,12 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>4.11</v>
+        <v>4.52</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -14264,14 +14274,14 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -14285,7 +14295,12 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>6.1</v>
+        <v>4.52</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -14294,14 +14309,14 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -14315,37 +14330,42 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6.1</v>
+        <v>4.52</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4.65</v>
+        <v>224</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -14354,42 +14374,822 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>kyaneos_pierre</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>224</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>kyaneos_pierre</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>224</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>210</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>210</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>210</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>682</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>682</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>682</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>pfo2</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>taux_distribution</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D74" t="n">
         <v>4.65</v>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G51"/>
+  <autoFilter ref="A1:G76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14400,7 +15200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14498,6 +15298,36 @@
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>corum_eurion</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
         </is>

</xml_diff>

<commit_message>
Collecte SCPI automatique 2026-09-21
</commit_message>
<xml_diff>
--- a/SCPI_tracker.xlsx
+++ b/SCPI_tracker.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparatif'!$A$1:$P$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sources'!$A$1:$H$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'A_VERIFIER'!$A$1:$E$234</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -908,7 +908,7 @@
     </comment>
     <comment ref="L11" authorId="0" shapeId="0">
       <text>
-        <t>Publié : 2026-06-30
+        <t>Publié : 2025-12-31
 Confiance : HAUTE
 Source : https://www.inter-gestion.com/offre-scpi/cristal-life</t>
       </text>
@@ -927,7 +927,7 @@
     </comment>
     <comment ref="C12" authorId="0" shapeId="0">
       <text>
-        <t>Publié : 2026-06-30
+        <t>Publié : 2025-12-31
 Confiance : HAUTE
 Source : https://www.inter-gestion.com/offre-scpi/cristal-rente</t>
       </text>
@@ -958,7 +958,7 @@
     </comment>
     <comment ref="J12" authorId="0" shapeId="0">
       <text>
-        <t>Publié : 2026-06-30
+        <t>Publié : 2025-12-31
 Confiance : HAUTE
 Source : https://www.inter-gestion.com/offre-scpi/cristal-rente</t>
       </text>
@@ -971,7 +971,7 @@
     </comment>
     <comment ref="L12" authorId="0" shapeId="0">
       <text>
-        <t>Publié : 2026-06-30
+        <t>Publié : 2025-12-31
 Confiance : HAUTE
 Source : https://www.inter-gestion.com/offre-scpi/cristal-rente</t>
       </text>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>225</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>699</v>
+        <v>932</v>
       </c>
     </row>
     <row r="16">
@@ -3246,7 +3246,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>424000000</v>
+        <v>387000000</v>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
@@ -3322,7 +3322,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>684000000</v>
+        <v>682000000</v>
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>424000000</v>
+        <v>387000000</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -6149,7 +6149,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>684000000</v>
+        <v>682000000</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -6158,7 +6158,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -6193,7 +6193,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -12739,7 +12739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12881,7 +12881,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>coeur_davenir</t>
+          <t>activimmo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -12890,11 +12890,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>200</v>
+        <v>613.5</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -12944,7 +12949,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -12956,7 +12961,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -12965,16 +12970,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>664</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -12986,7 +12986,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -12995,16 +12995,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>664</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -13034,7 +13029,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -13051,16 +13046,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -13086,16 +13076,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -13104,7 +13089,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -13121,16 +13106,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -13139,7 +13119,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -13151,16 +13131,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -13181,16 +13166,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -13211,16 +13201,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -13241,7 +13236,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -13255,7 +13250,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6.25</v>
+        <v>6.2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -13264,7 +13259,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -13281,16 +13276,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -13316,16 +13306,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -13334,7 +13319,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -13346,7 +13331,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -13355,7 +13340,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -13364,7 +13349,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -13376,7 +13361,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -13385,7 +13370,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -13394,7 +13379,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -13406,16 +13391,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -13424,7 +13414,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -13436,7 +13426,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -13450,7 +13440,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -13471,7 +13461,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -13485,7 +13475,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -13494,7 +13484,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -13506,7 +13496,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -13520,7 +13510,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -13529,7 +13519,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -13541,21 +13531,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>acompte</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2.75</v>
+        <v>250</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -13576,21 +13561,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>acompte</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2.75</v>
+        <v>250</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -13611,21 +13591,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>acompte</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.75</v>
+        <v>250</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -13646,7 +13621,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -13654,13 +13629,8 @@
           <t>prix_souscription</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
-        </is>
-      </c>
       <c r="D29" t="n">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -13669,33 +13639,33 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>215</v>
+        <v>6</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -13709,28 +13679,28 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>215</v>
+        <v>6</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -13739,19 +13709,19 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -13765,7 +13735,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>5.73</v>
+        <v>6</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -13774,7 +13744,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -13786,7 +13756,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -13800,7 +13770,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>5.73</v>
+        <v>6</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -13809,7 +13779,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13826,16 +13796,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -13844,7 +13814,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -13856,12 +13826,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -13870,7 +13840,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>200</v>
+        <v>2.75</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -13884,19 +13854,19 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -13905,7 +13875,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>200</v>
+        <v>2.75</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -13914,24 +13884,24 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -13940,7 +13910,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>200</v>
+        <v>2.75</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -13949,33 +13919,33 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>7.7</v>
+        <v>215</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -13989,28 +13959,28 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>7.7</v>
+        <v>215</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -14024,28 +13994,28 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>7.7</v>
+        <v>215</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -14059,14 +14029,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -14074,8 +14044,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D41" t="n">
-        <v>255.68</v>
+        <v>215</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -14084,28 +14059,33 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>255.68</v>
+        <v>5.73</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -14126,16 +14106,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>255.68</v>
+        <v>5.73</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -14144,7 +14129,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -14156,16 +14141,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>202</v>
+        <v>5.73</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -14174,7 +14164,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -14186,16 +14176,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>202</v>
+        <v>5.73</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -14204,7 +14199,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -14216,7 +14211,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -14224,8 +14219,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D46" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -14234,33 +14234,33 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>4.52</v>
+        <v>200</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -14274,28 +14274,28 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>4.52</v>
+        <v>200</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -14304,33 +14304,33 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>4.52</v>
+        <v>200</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -14339,28 +14339,33 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>224</v>
+        <v>7.7</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -14381,16 +14386,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>224</v>
+        <v>7.7</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -14411,16 +14421,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>224</v>
+        <v>7.7</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -14441,16 +14456,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>210</v>
+        <v>7.7</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -14459,7 +14479,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -14471,7 +14491,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -14480,7 +14500,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>210</v>
+        <v>255.68</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -14501,7 +14521,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -14510,7 +14530,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>210</v>
+        <v>255.68</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -14519,7 +14539,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -14531,21 +14551,16 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>7.1</v>
+        <v>255.68</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -14554,7 +14569,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -14566,30 +14581,25 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>7.1</v>
+        <v>255.68</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -14601,21 +14611,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>7.1</v>
+        <v>202</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -14624,7 +14629,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -14636,7 +14641,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -14645,7 +14650,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>682</v>
+        <v>202</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -14666,7 +14671,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -14675,7 +14680,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>682</v>
+        <v>202</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -14684,7 +14689,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -14696,7 +14701,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -14705,7 +14710,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>682</v>
+        <v>202</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -14714,7 +14719,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -14726,7 +14731,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -14740,7 +14745,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7.51</v>
+        <v>4.52</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -14761,7 +14766,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -14775,7 +14780,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>7.51</v>
+        <v>4.52</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -14796,7 +14801,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -14810,7 +14815,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>7.51</v>
+        <v>4.52</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -14831,7 +14836,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -14845,37 +14850,42 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>4.8</v>
+        <v>4.52</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>4.8</v>
+        <v>224</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -14884,148 +14894,148 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>4.8</v>
+        <v>224</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>4.11</v>
+        <v>224</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>4.11</v>
+        <v>224</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4.11</v>
+        <v>210</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>6.1</v>
+        <v>210</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -15034,74 +15044,74 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>6.1</v>
+        <v>210</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>6.1</v>
+        <v>210</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -15115,7 +15125,12 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>4.65</v>
+        <v>7.1</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -15124,14 +15139,14 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -15145,7 +15160,12 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>4.65</v>
+        <v>7.1</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -15154,42 +15174,822 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ncap_continent</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>682</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>682</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>682</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>prix_souscription</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>682</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
           <t>pfo2</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>taux_distribution</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D76" t="n">
+      <c r="D98" t="n">
         <v>4.65</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F100" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G100" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G76"/>
+  <autoFilter ref="A1:G101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15200,7 +16000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -15328,6 +16128,36 @@
         </is>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>corum_eurion</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
         </is>

</xml_diff>

<commit_message>
Collecte SCPI automatique 2026-10-05
</commit_message>
<xml_diff>
--- a/SCPI_tracker.xlsx
+++ b/SCPI_tracker.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparatif'!$A$1:$P$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sources'!$A$1:$H$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'A_VERIFIER'!$A$1:$E$236</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>375</v>
+        <v>450</v>
       </c>
     </row>
     <row r="13">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1143</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="16">
@@ -12783,7 +12783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12985,7 +12985,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>coeur_davenir</t>
+          <t>activimmo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -12994,11 +12994,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>200</v>
+        <v>613.5</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -13048,7 +13053,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -13073,7 +13078,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -13098,7 +13103,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -13110,7 +13115,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -13119,16 +13124,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>664</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -13140,7 +13140,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -13149,16 +13149,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>664</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -13188,7 +13183,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -13218,7 +13213,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -13248,7 +13243,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -13265,16 +13260,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -13283,7 +13273,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -13300,16 +13290,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -13318,7 +13303,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -13335,16 +13320,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -13353,7 +13333,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -13388,7 +13368,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -13423,7 +13403,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -13435,16 +13415,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -13453,7 +13438,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -13465,16 +13450,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -13483,7 +13473,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -13495,16 +13485,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -13513,7 +13508,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -13525,16 +13520,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -13543,7 +13543,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -13573,7 +13573,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -13590,16 +13590,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -13625,16 +13620,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -13643,7 +13633,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -13660,16 +13650,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -13678,7 +13663,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -13695,16 +13680,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -13713,7 +13693,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -13730,16 +13710,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -13748,7 +13723,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -13760,16 +13735,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -13790,16 +13770,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -13820,16 +13805,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -13850,16 +13840,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -13880,16 +13875,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -13910,7 +13910,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -13924,7 +13924,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -13933,7 +13933,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -13950,16 +13950,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -13985,16 +13980,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -14003,7 +13993,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -14020,16 +14010,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -14038,7 +14023,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -14055,16 +14040,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -14073,7 +14053,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -14085,21 +14065,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>acompte</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2.75</v>
+        <v>250</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -14108,7 +14083,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -14120,21 +14095,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>acompte</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2.75</v>
+        <v>250</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -14143,7 +14113,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -14155,21 +14125,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -14178,7 +14148,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -14190,21 +14160,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -14213,7 +14183,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -14225,21 +14195,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -14248,7 +14218,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -14260,21 +14230,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>215</v>
+        <v>6</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -14283,33 +14253,33 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>215</v>
+        <v>6</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -14318,33 +14288,33 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>215</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -14353,12 +14323,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14370,7 +14340,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -14379,7 +14349,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>215</v>
+        <v>2.75</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -14388,12 +14358,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14405,7 +14375,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -14414,7 +14384,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>215</v>
+        <v>2.75</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -14423,12 +14393,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14440,16 +14410,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -14458,7 +14428,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -14475,16 +14445,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -14493,7 +14463,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -14510,16 +14480,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -14528,7 +14498,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -14545,16 +14515,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -14563,7 +14533,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -14580,16 +14550,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5.73</v>
+        <v>215</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -14598,19 +14568,19 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -14624,7 +14594,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -14645,7 +14615,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -14659,7 +14629,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -14668,7 +14638,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -14680,7 +14650,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -14694,7 +14664,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -14703,7 +14673,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -14715,7 +14685,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -14729,7 +14699,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -14738,7 +14708,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -14750,7 +14720,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -14764,7 +14734,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -14773,7 +14743,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -14785,7 +14755,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -14799,7 +14769,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -14820,7 +14790,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -14834,7 +14804,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -14855,7 +14825,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -14869,7 +14839,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -14890,7 +14860,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -14904,7 +14874,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -14925,7 +14895,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -14939,7 +14909,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -14960,16 +14930,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>255.68</v>
+        <v>5.73</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -14978,7 +14953,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -14990,7 +14965,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -14998,8 +14973,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D68" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -15013,14 +14993,14 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -15028,8 +15008,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D69" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -15038,19 +15023,19 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -15058,29 +15043,34 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D70" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -15088,29 +15078,34 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D71" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -15118,8 +15113,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D72" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -15128,19 +15128,19 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -15148,8 +15148,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D73" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -15158,28 +15163,33 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -15188,7 +15198,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -15200,16 +15210,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -15218,7 +15233,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -15230,16 +15245,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -15248,7 +15268,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -15260,7 +15280,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -15274,7 +15294,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>4.52</v>
+        <v>7.7</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -15283,7 +15303,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -15295,7 +15315,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -15309,7 +15329,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>4.52</v>
+        <v>7.7</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -15318,7 +15338,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -15330,7 +15350,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -15344,7 +15364,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>4.52</v>
+        <v>7.7</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -15353,7 +15373,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -15365,21 +15385,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>4.52</v>
+        <v>255.68</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -15388,7 +15403,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -15400,21 +15415,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>4.52</v>
+        <v>255.68</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -15423,7 +15433,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -15435,7 +15445,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -15444,7 +15454,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>224</v>
+        <v>255.68</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -15453,7 +15463,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -15465,7 +15475,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -15474,16 +15484,16 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>224</v>
+        <v>255.68</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -15495,7 +15505,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -15504,16 +15514,16 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>224</v>
+        <v>255.68</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -15525,7 +15535,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -15534,16 +15544,16 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>224</v>
+        <v>255.68</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -15555,7 +15565,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -15564,7 +15574,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -15573,7 +15583,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -15585,7 +15595,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -15594,7 +15604,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -15615,7 +15625,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -15624,7 +15634,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -15633,7 +15643,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -15645,7 +15655,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -15654,7 +15664,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -15663,7 +15673,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -15675,7 +15685,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -15684,7 +15694,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -15693,7 +15703,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -15705,7 +15715,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -15714,7 +15724,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -15723,7 +15733,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -15735,7 +15745,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -15749,7 +15759,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -15770,7 +15780,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -15784,7 +15794,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -15805,7 +15815,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -15819,7 +15829,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -15840,7 +15850,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -15854,7 +15864,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -15875,7 +15885,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -15889,7 +15899,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -15910,16 +15920,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>682</v>
+        <v>4.52</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -15928,7 +15943,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -15940,7 +15955,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -15949,7 +15964,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -15970,7 +15985,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -15979,7 +15994,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -15988,7 +16003,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -16000,7 +16015,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -16009,7 +16024,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -16018,7 +16033,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -16030,7 +16045,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -16039,7 +16054,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -16048,7 +16063,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -16060,21 +16075,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>7.51</v>
+        <v>224</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -16083,7 +16093,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -16095,21 +16105,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>7.51</v>
+        <v>224</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -16118,7 +16123,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -16130,21 +16135,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -16153,7 +16153,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -16165,21 +16165,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -16188,7 +16183,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -16200,21 +16195,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -16223,7 +16213,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -16235,97 +16225,97 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>4.8</v>
+        <v>210</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>4.8</v>
+        <v>210</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>4.8</v>
+        <v>210</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -16339,23 +16329,28 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -16369,23 +16364,28 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -16399,23 +16399,28 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>4.11</v>
+        <v>7.1</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -16429,23 +16434,28 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>4.11</v>
+        <v>7.1</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -16459,23 +16469,28 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>4.11</v>
+        <v>7.1</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -16489,67 +16504,72 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>4.11</v>
+        <v>7.1</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>4.11</v>
+        <v>682</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>6.1</v>
+        <v>682</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -16558,134 +16578,134 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>6.1</v>
+        <v>682</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>6.1</v>
+        <v>682</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>6.1</v>
+        <v>682</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>6.1</v>
+        <v>682</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -16699,7 +16719,12 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>4.65</v>
+        <v>7.51</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -16708,14 +16733,14 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -16729,7 +16754,12 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>4.65</v>
+        <v>7.51</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -16738,14 +16768,14 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -16759,7 +16789,12 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>4.65</v>
+        <v>7.51</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -16768,14 +16803,14 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -16789,7 +16824,12 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>4.65</v>
+        <v>7.51</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -16798,42 +16838,802 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>ncap_regions</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
           <t>pfo2</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B146" t="inlineStr">
         <is>
           <t>taux_distribution</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C146" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D126" t="n">
+      <c r="D146" t="n">
         <v>4.65</v>
       </c>
-      <c r="F126" t="inlineStr">
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F150" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr">
+      <c r="G150" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G126"/>
+  <autoFilter ref="A1:G151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16844,7 +17644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -17032,6 +17832,36 @@
         </is>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>corum_eurion</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
         </is>

</xml_diff>

<commit_message>
Collecte SCPI automatique 2026-10-12
</commit_message>
<xml_diff>
--- a/SCPI_tracker.xlsx
+++ b/SCPI_tracker.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparatif'!$A$1:$P$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sources'!$A$1:$H$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'A_VERIFIER'!$A$1:$E$236</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historique'!$A$1:$G$176</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>450</v>
+        <v>525</v>
       </c>
     </row>
     <row r="13">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1376</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="16">
@@ -12783,7 +12783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G151"/>
+  <dimension ref="A1:G176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13015,7 +13015,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>coeur_davenir</t>
+          <t>activimmo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -13024,11 +13024,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>200</v>
+        <v>613.5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -13078,7 +13083,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -13103,7 +13108,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -13128,7 +13133,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -13153,7 +13158,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -13165,7 +13170,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -13174,16 +13179,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>664</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -13195,7 +13195,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>coeur_de_regions</t>
+          <t>coeur_davenir</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -13204,16 +13204,11 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>664</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
+        <v>200</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -13243,7 +13238,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -13273,7 +13268,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -13303,7 +13298,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -13333,7 +13328,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -13350,16 +13345,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -13368,7 +13358,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -13385,16 +13375,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -13403,7 +13388,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -13420,16 +13405,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6.2</v>
+        <v>664</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -13438,7 +13418,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -13473,7 +13453,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -13508,7 +13488,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -13543,7 +13523,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -13555,16 +13535,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -13573,7 +13558,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -13585,16 +13570,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -13603,7 +13593,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -13615,16 +13605,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -13633,7 +13628,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -13645,16 +13640,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>coeur_deurope</t>
+          <t>coeur_de_regions</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>204</v>
+        <v>6.2</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -13663,7 +13663,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -13693,7 +13693,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -13723,7 +13723,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -13740,16 +13740,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -13758,7 +13753,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -13775,16 +13770,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -13793,7 +13783,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -13810,16 +13800,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -13828,7 +13813,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -13845,16 +13830,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -13863,7 +13843,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13880,16 +13860,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>6.25</v>
+        <v>204</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -13898,7 +13873,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -13933,7 +13908,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -13945,16 +13920,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -13975,16 +13955,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -13993,7 +13978,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -14005,16 +13990,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -14023,7 +14013,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -14035,16 +14025,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -14053,7 +14048,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -14065,16 +14060,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -14083,7 +14083,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -14095,16 +14095,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>comete</t>
+          <t>coeur_deurope</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>250</v>
+        <v>6.25</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -14113,7 +14118,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -14130,16 +14135,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -14165,16 +14165,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -14200,16 +14195,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -14235,16 +14225,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -14270,16 +14255,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -14305,16 +14285,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>250</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -14335,21 +14310,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>acompte</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>2026-T2</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2.75</v>
+        <v>250</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -14358,7 +14328,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -14370,21 +14340,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -14405,21 +14375,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -14428,7 +14398,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -14440,21 +14410,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -14463,7 +14433,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -14475,21 +14445,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -14498,7 +14468,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -14510,21 +14480,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>acompte</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -14533,7 +14503,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -14545,21 +14515,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>215</v>
+        <v>6</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -14568,33 +14538,33 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>corum_eurion</t>
+          <t>comete</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>215</v>
+        <v>6</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -14603,12 +14573,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14620,7 +14590,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -14629,7 +14599,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>215</v>
+        <v>2.75</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -14638,12 +14608,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14655,7 +14625,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -14664,7 +14634,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>215</v>
+        <v>2.75</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -14673,12 +14643,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14690,7 +14660,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -14699,7 +14669,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>215</v>
+        <v>2.75</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -14708,12 +14678,12 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14725,7 +14695,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -14734,7 +14704,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>215</v>
+        <v>2.75</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -14743,12 +14713,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
@@ -14760,16 +14730,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -14778,7 +14748,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -14795,16 +14765,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -14813,7 +14783,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -14830,16 +14800,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>acompte</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5.73</v>
+        <v>2.75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -14848,7 +14818,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -14865,16 +14835,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>5.73</v>
+        <v>215</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -14883,12 +14853,12 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
@@ -14900,16 +14870,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>5.73</v>
+        <v>215</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -14918,12 +14888,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
@@ -14935,16 +14905,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5.73</v>
+        <v>215</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -14953,19 +14923,19 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -14979,7 +14949,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -14988,7 +14958,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -15000,7 +14970,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -15014,7 +14984,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -15023,7 +14993,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -15035,7 +15005,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -15049,7 +15019,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -15058,7 +15028,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -15070,7 +15040,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -15084,7 +15054,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -15093,7 +15063,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -15105,21 +15075,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>200</v>
+        <v>5.73</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -15128,33 +15098,33 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-T2</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>200</v>
+        <v>5.73</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -15163,19 +15133,19 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -15189,7 +15159,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -15198,7 +15168,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -15210,7 +15180,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -15224,7 +15194,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -15233,7 +15203,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -15245,7 +15215,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -15259,7 +15229,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -15268,7 +15238,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -15280,7 +15250,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -15294,7 +15264,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -15303,7 +15273,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -15315,7 +15285,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>corum_usa</t>
+          <t>corum_eurion</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -15329,7 +15299,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>7.7</v>
+        <v>5.73</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -15338,7 +15308,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -15355,16 +15325,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-T2</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>7.7</v>
+        <v>200</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -15373,19 +15343,19 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -15393,8 +15363,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D80" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -15408,14 +15383,14 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -15423,8 +15398,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D81" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -15433,19 +15413,19 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -15453,8 +15433,13 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D82" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -15463,19 +15448,19 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -15483,29 +15468,34 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D83" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -15513,29 +15503,34 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D84" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>cristal_rente</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -15543,38 +15538,48 @@
           <t>prix_souscription</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
       <c r="D85" t="n">
-        <v>255.68</v>
+        <v>200</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>HAUTE</t>
+          <t>MOYENNE</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -15595,16 +15600,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -15625,16 +15635,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -15655,16 +15670,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -15685,16 +15705,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -15715,16 +15740,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>202</v>
+        <v>7.7</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -15745,7 +15775,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>corum_usa</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -15759,7 +15789,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>4.52</v>
+        <v>7.7</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -15768,7 +15798,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -15780,21 +15810,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>4.52</v>
+        <v>255.68</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -15815,21 +15840,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>4.52</v>
+        <v>255.68</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -15838,7 +15858,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -15850,21 +15870,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>4.52</v>
+        <v>255.68</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -15873,7 +15888,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -15885,30 +15900,25 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>4.52</v>
+        <v>255.68</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -15920,30 +15930,25 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>fair_invest</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>4.52</v>
+        <v>255.68</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -15955,7 +15960,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -15964,16 +15969,16 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>224</v>
+        <v>255.68</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -15985,7 +15990,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>cristal_rente</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -15994,16 +15999,16 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>224</v>
+        <v>255.68</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -16015,7 +16020,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -16024,7 +16029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -16033,7 +16038,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -16045,7 +16050,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -16054,7 +16059,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -16063,7 +16068,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -16075,7 +16080,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -16084,7 +16089,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -16093,7 +16098,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -16105,7 +16110,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>kyaneos_pierre</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -16114,7 +16119,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -16123,7 +16128,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -16135,7 +16140,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -16144,7 +16149,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -16153,7 +16158,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -16165,7 +16170,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -16174,7 +16179,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -16183,7 +16188,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -16195,7 +16200,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -16204,7 +16209,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -16213,7 +16218,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -16225,16 +16230,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>210</v>
+        <v>4.52</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -16243,7 +16253,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -16255,16 +16265,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>210</v>
+        <v>4.52</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -16273,7 +16288,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -16285,16 +16300,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>prix_souscription</t>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>210</v>
+        <v>4.52</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -16303,7 +16323,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -16315,7 +16335,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -16329,7 +16349,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -16338,7 +16358,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -16350,7 +16370,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -16364,7 +16384,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -16373,7 +16393,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -16385,7 +16405,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -16399,7 +16419,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -16408,7 +16428,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -16420,7 +16440,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>fair_invest</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -16434,7 +16454,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>7.1</v>
+        <v>4.52</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -16443,7 +16463,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -16455,21 +16475,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>7.1</v>
+        <v>224</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -16478,7 +16493,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -16490,21 +16505,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ncap_continent</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>7.1</v>
+        <v>224</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -16513,7 +16523,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -16525,7 +16535,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -16534,7 +16544,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -16543,7 +16553,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -16555,7 +16565,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -16564,7 +16574,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -16573,7 +16583,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -16585,7 +16595,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -16594,7 +16604,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -16603,7 +16613,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -16615,7 +16625,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -16624,7 +16634,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -16633,7 +16643,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -16645,7 +16655,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>kyaneos_pierre</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -16654,7 +16664,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>682</v>
+        <v>224</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -16663,7 +16673,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -16675,7 +16685,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -16684,7 +16694,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>682</v>
+        <v>210</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -16693,7 +16703,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -16705,21 +16715,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -16740,21 +16745,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -16763,7 +16763,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -16775,21 +16775,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -16798,7 +16793,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -16810,21 +16805,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -16833,7 +16823,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -16845,21 +16835,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -16868,7 +16853,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -16880,21 +16865,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ncap_regions</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>7.51</v>
+        <v>210</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -16903,7 +16883,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -16915,7 +16895,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -16929,7 +16909,12 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -16938,14 +16923,14 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -16959,7 +16944,12 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -16968,14 +16958,14 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -16989,7 +16979,12 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -16998,14 +16993,14 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -17019,7 +17014,12 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -17028,14 +17028,14 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -17049,7 +17049,12 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -17058,14 +17063,14 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>pf_grand_paris</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -17079,7 +17084,12 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>4.8</v>
+        <v>7.1</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -17088,14 +17098,14 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_continent</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -17109,37 +17119,42 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>4.11</v>
+        <v>7.1</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>4.11</v>
+        <v>682</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -17148,194 +17163,194 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4.11</v>
+        <v>682</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4.11</v>
+        <v>682</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>4.11</v>
+        <v>682</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>pf_hospitalite_europe</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>4.11</v>
+        <v>682</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>6.1</v>
+        <v>682</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>taux_distribution</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>prix_souscription</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>6.1</v>
+        <v>682</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -17349,23 +17364,28 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>6.1</v>
+        <v>7.51</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -17379,23 +17399,28 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>6.1</v>
+        <v>7.51</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -17409,23 +17434,28 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>6.1</v>
+        <v>7.51</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>pfo</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -17439,23 +17469,28 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>6.1</v>
+        <v>7.51</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -17469,23 +17504,28 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>4.65</v>
+        <v>7.51</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -17499,23 +17539,28 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>4.65</v>
+        <v>7.51</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>ncap_regions</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -17529,23 +17574,28 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>4.65</v>
+        <v>7.51</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>MOYENNE</t>
+          <t>HAUTE</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>pf_grand_paris</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -17559,11 +17609,11 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>4.65</v>
+        <v>4.8</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -17575,7 +17625,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>pfo2</t>
+          <t>pf_grand_paris</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -17589,11 +17639,11 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>4.65</v>
+        <v>4.8</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -17605,35 +17655,785 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>pf_grand_paris</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>pf_hospitalite_europe</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>pfo</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
           <t>pfo2</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B170" t="inlineStr">
         <is>
           <t>taux_distribution</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C170" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D151" t="n">
+      <c r="D170" t="n">
         <v>4.65</v>
       </c>
-      <c r="F151" t="inlineStr">
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F175" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr">
+      <c r="G175" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>pfo2</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>taux_distribution</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G151"/>
+  <autoFilter ref="A1:G176"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17644,7 +18444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -17862,6 +18662,36 @@
         </is>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>corum_eurion</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-T2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://www.corum.fr/sites/default/files/2026-07/CORUM%20Eurion%20-%20Fil%20d%27Actualit%C3%A9s%202026-T2.pdf</t>
         </is>

</xml_diff>